<commit_message>
updated week daze poll results
</commit_message>
<xml_diff>
--- a/whiteboardpollresults.xlsx
+++ b/whiteboardpollresults.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mbrownin\GitHub - Local\thehallwaypoll\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C3F21C0-06F8-499A-B908-312602C41141}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD209EB1-B4D5-4541-A45E-C12722BD993B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="686" xr2:uid="{C0D0DBC0-4258-4C8D-AB0A-404DBED773F9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="804" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="303">
   <si>
     <t>option</t>
   </si>
@@ -891,6 +891,60 @@
   </si>
   <si>
     <t>Longest-Feeling</t>
+  </si>
+  <si>
+    <t>Labor of Love?</t>
+  </si>
+  <si>
+    <t>Left</t>
+  </si>
+  <si>
+    <t>Right</t>
+  </si>
+  <si>
+    <t>EISD Tickets</t>
+  </si>
+  <si>
+    <t>Submit immediately</t>
+  </si>
+  <si>
+    <t>Wait until its really a problem</t>
+  </si>
+  <si>
+    <t>Cube Farm Traffic</t>
+  </si>
+  <si>
+    <t>Teams Meetings</t>
+  </si>
+  <si>
+    <t>Join right on time</t>
+  </si>
+  <si>
+    <t>Start a few minutes early</t>
+  </si>
+  <si>
+    <t>Worst Office Temperature</t>
+  </si>
+  <si>
+    <t>Too Hot</t>
+  </si>
+  <si>
+    <t>Too Cold</t>
+  </si>
+  <si>
+    <t>Best Email Signoff</t>
+  </si>
+  <si>
+    <t>Thanks</t>
+  </si>
+  <si>
+    <t>Sincerely</t>
+  </si>
+  <si>
+    <t>Cheers</t>
+  </si>
+  <si>
+    <t>Best</t>
   </si>
 </sst>
 </file>
@@ -1263,7 +1317,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C897EEBF-8298-48F4-84CA-7840A621B809}">
-  <dimension ref="A1:H200"/>
+  <dimension ref="A1:H212"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
@@ -5533,7 +5587,7 @@
         <v>273</v>
       </c>
       <c r="C173" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D173" t="s">
         <v>281</v>
@@ -5541,8 +5595,14 @@
       <c r="E173" t="s">
         <v>274</v>
       </c>
+      <c r="F173">
+        <v>1</v>
+      </c>
+      <c r="G173">
+        <v>3</v>
+      </c>
       <c r="H173" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="174" spans="1:8" x14ac:dyDescent="0.25">
@@ -5553,7 +5613,7 @@
         <v>273</v>
       </c>
       <c r="C174" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D174" t="s">
         <v>281</v>
@@ -5561,8 +5621,14 @@
       <c r="E174" t="s">
         <v>275</v>
       </c>
+      <c r="F174">
+        <v>3</v>
+      </c>
+      <c r="G174">
+        <v>1</v>
+      </c>
       <c r="H174" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="175" spans="1:8" x14ac:dyDescent="0.25">
@@ -5573,7 +5639,7 @@
         <v>273</v>
       </c>
       <c r="C175" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D175" t="s">
         <v>281</v>
@@ -5581,8 +5647,14 @@
       <c r="E175" t="s">
         <v>276</v>
       </c>
+      <c r="F175">
+        <v>1</v>
+      </c>
+      <c r="G175">
+        <v>0</v>
+      </c>
       <c r="H175" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="176" spans="1:8" x14ac:dyDescent="0.25">
@@ -5593,7 +5665,7 @@
         <v>273</v>
       </c>
       <c r="C176" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D176" t="s">
         <v>281</v>
@@ -5601,8 +5673,14 @@
       <c r="E176" t="s">
         <v>277</v>
       </c>
+      <c r="F176">
+        <v>4</v>
+      </c>
+      <c r="G176">
+        <v>0</v>
+      </c>
       <c r="H176" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="177" spans="1:8" x14ac:dyDescent="0.25">
@@ -5613,7 +5691,7 @@
         <v>273</v>
       </c>
       <c r="C177" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D177" t="s">
         <v>281</v>
@@ -5621,8 +5699,14 @@
       <c r="E177" t="s">
         <v>278</v>
       </c>
+      <c r="F177">
+        <v>20</v>
+      </c>
+      <c r="G177">
+        <v>5</v>
+      </c>
       <c r="H177" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="178" spans="1:8" x14ac:dyDescent="0.25">
@@ -5633,7 +5717,7 @@
         <v>273</v>
       </c>
       <c r="C178" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D178" t="s">
         <v>281</v>
@@ -5641,8 +5725,14 @@
       <c r="E178" t="s">
         <v>279</v>
       </c>
+      <c r="F178">
+        <v>29</v>
+      </c>
+      <c r="G178">
+        <v>19</v>
+      </c>
       <c r="H178" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="179" spans="1:8" x14ac:dyDescent="0.25">
@@ -5653,7 +5743,7 @@
         <v>273</v>
       </c>
       <c r="C179" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D179" t="s">
         <v>281</v>
@@ -5661,8 +5751,14 @@
       <c r="E179" t="s">
         <v>280</v>
       </c>
+      <c r="F179">
+        <v>2</v>
+      </c>
+      <c r="G179">
+        <v>4</v>
+      </c>
       <c r="H179" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="180" spans="1:8" x14ac:dyDescent="0.25">
@@ -5673,7 +5769,7 @@
         <v>273</v>
       </c>
       <c r="C180" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D180" t="s">
         <v>282</v>
@@ -5681,8 +5777,14 @@
       <c r="E180" t="s">
         <v>274</v>
       </c>
+      <c r="F180">
+        <v>28</v>
+      </c>
+      <c r="G180">
+        <v>15</v>
+      </c>
       <c r="H180" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="181" spans="1:8" x14ac:dyDescent="0.25">
@@ -5693,7 +5795,7 @@
         <v>273</v>
       </c>
       <c r="C181" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D181" t="s">
         <v>282</v>
@@ -5701,8 +5803,14 @@
       <c r="E181" t="s">
         <v>275</v>
       </c>
+      <c r="F181">
+        <v>13</v>
+      </c>
+      <c r="G181">
+        <v>7</v>
+      </c>
       <c r="H181" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="182" spans="1:8" x14ac:dyDescent="0.25">
@@ -5713,7 +5821,7 @@
         <v>273</v>
       </c>
       <c r="C182" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D182" t="s">
         <v>282</v>
@@ -5721,8 +5829,14 @@
       <c r="E182" t="s">
         <v>276</v>
       </c>
+      <c r="F182">
+        <v>3</v>
+      </c>
+      <c r="G182">
+        <v>6</v>
+      </c>
       <c r="H182" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="183" spans="1:8" x14ac:dyDescent="0.25">
@@ -5733,7 +5847,7 @@
         <v>273</v>
       </c>
       <c r="C183" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D183" t="s">
         <v>282</v>
@@ -5741,8 +5855,14 @@
       <c r="E183" t="s">
         <v>277</v>
       </c>
+      <c r="F183">
+        <v>5</v>
+      </c>
+      <c r="G183">
+        <v>3</v>
+      </c>
       <c r="H183" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="184" spans="1:8" x14ac:dyDescent="0.25">
@@ -5753,7 +5873,7 @@
         <v>273</v>
       </c>
       <c r="C184" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D184" t="s">
         <v>282</v>
@@ -5761,8 +5881,14 @@
       <c r="E184" t="s">
         <v>278</v>
       </c>
+      <c r="F184">
+        <v>0</v>
+      </c>
+      <c r="G184">
+        <v>1</v>
+      </c>
       <c r="H184" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="185" spans="1:8" x14ac:dyDescent="0.25">
@@ -5773,7 +5899,7 @@
         <v>273</v>
       </c>
       <c r="C185" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D185" t="s">
         <v>282</v>
@@ -5781,8 +5907,14 @@
       <c r="E185" t="s">
         <v>279</v>
       </c>
+      <c r="F185">
+        <v>0</v>
+      </c>
+      <c r="G185">
+        <v>0</v>
+      </c>
       <c r="H185" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="186" spans="1:8" x14ac:dyDescent="0.25">
@@ -5793,7 +5925,7 @@
         <v>273</v>
       </c>
       <c r="C186" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D186" t="s">
         <v>282</v>
@@ -5801,8 +5933,14 @@
       <c r="E186" t="s">
         <v>280</v>
       </c>
+      <c r="F186">
+        <v>5</v>
+      </c>
+      <c r="G186">
+        <v>0</v>
+      </c>
       <c r="H186" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="187" spans="1:8" x14ac:dyDescent="0.25">
@@ -5813,7 +5951,7 @@
         <v>273</v>
       </c>
       <c r="C187" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D187" t="s">
         <v>283</v>
@@ -5821,8 +5959,14 @@
       <c r="E187" t="s">
         <v>274</v>
       </c>
+      <c r="F187">
+        <v>9</v>
+      </c>
+      <c r="G187">
+        <v>2</v>
+      </c>
       <c r="H187" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="188" spans="1:8" x14ac:dyDescent="0.25">
@@ -5833,7 +5977,7 @@
         <v>273</v>
       </c>
       <c r="C188" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D188" t="s">
         <v>283</v>
@@ -5841,8 +5985,14 @@
       <c r="E188" t="s">
         <v>275</v>
       </c>
+      <c r="F188">
+        <v>14</v>
+      </c>
+      <c r="G188">
+        <v>10</v>
+      </c>
       <c r="H188" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="189" spans="1:8" x14ac:dyDescent="0.25">
@@ -5853,7 +6003,7 @@
         <v>273</v>
       </c>
       <c r="C189" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D189" t="s">
         <v>283</v>
@@ -5861,8 +6011,14 @@
       <c r="E189" t="s">
         <v>276</v>
       </c>
+      <c r="F189">
+        <v>16</v>
+      </c>
+      <c r="G189">
+        <v>5</v>
+      </c>
       <c r="H189" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="190" spans="1:8" x14ac:dyDescent="0.25">
@@ -5873,7 +6029,7 @@
         <v>273</v>
       </c>
       <c r="C190" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D190" t="s">
         <v>283</v>
@@ -5881,8 +6037,14 @@
       <c r="E190" t="s">
         <v>277</v>
       </c>
+      <c r="F190">
+        <v>14</v>
+      </c>
+      <c r="G190">
+        <v>7</v>
+      </c>
       <c r="H190" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="191" spans="1:8" x14ac:dyDescent="0.25">
@@ -5893,7 +6055,7 @@
         <v>273</v>
       </c>
       <c r="C191" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D191" t="s">
         <v>283</v>
@@ -5901,8 +6063,14 @@
       <c r="E191" t="s">
         <v>278</v>
       </c>
+      <c r="F191">
+        <v>5</v>
+      </c>
+      <c r="G191">
+        <v>6</v>
+      </c>
       <c r="H191" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="192" spans="1:8" x14ac:dyDescent="0.25">
@@ -5913,7 +6081,7 @@
         <v>273</v>
       </c>
       <c r="C192" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D192" t="s">
         <v>283</v>
@@ -5921,8 +6089,14 @@
       <c r="E192" t="s">
         <v>279</v>
       </c>
+      <c r="F192">
+        <v>2</v>
+      </c>
+      <c r="G192">
+        <v>0</v>
+      </c>
       <c r="H192" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="193" spans="1:8" x14ac:dyDescent="0.25">
@@ -5933,7 +6107,7 @@
         <v>273</v>
       </c>
       <c r="C193" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D193" t="s">
         <v>283</v>
@@ -5941,8 +6115,14 @@
       <c r="E193" t="s">
         <v>280</v>
       </c>
+      <c r="F193">
+        <v>0</v>
+      </c>
+      <c r="G193">
+        <v>3</v>
+      </c>
       <c r="H193" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="194" spans="1:8" x14ac:dyDescent="0.25">
@@ -5953,7 +6133,7 @@
         <v>273</v>
       </c>
       <c r="C194" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D194" t="s">
         <v>284</v>
@@ -5961,8 +6141,14 @@
       <c r="E194" t="s">
         <v>274</v>
       </c>
+      <c r="F194">
+        <v>10</v>
+      </c>
+      <c r="G194">
+        <v>4</v>
+      </c>
       <c r="H194" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="195" spans="1:8" x14ac:dyDescent="0.25">
@@ -5973,7 +6159,7 @@
         <v>273</v>
       </c>
       <c r="C195" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D195" t="s">
         <v>284</v>
@@ -5981,8 +6167,14 @@
       <c r="E195" t="s">
         <v>275</v>
       </c>
+      <c r="F195">
+        <v>13</v>
+      </c>
+      <c r="G195">
+        <v>10</v>
+      </c>
       <c r="H195" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="196" spans="1:8" x14ac:dyDescent="0.25">
@@ -5993,7 +6185,7 @@
         <v>273</v>
       </c>
       <c r="C196" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D196" t="s">
         <v>284</v>
@@ -6001,8 +6193,14 @@
       <c r="E196" t="s">
         <v>276</v>
       </c>
+      <c r="F196">
+        <v>15</v>
+      </c>
+      <c r="G196">
+        <v>8</v>
+      </c>
       <c r="H196" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="197" spans="1:8" x14ac:dyDescent="0.25">
@@ -6013,7 +6211,7 @@
         <v>273</v>
       </c>
       <c r="C197" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D197" t="s">
         <v>284</v>
@@ -6021,8 +6219,14 @@
       <c r="E197" t="s">
         <v>277</v>
       </c>
+      <c r="F197">
+        <v>17</v>
+      </c>
+      <c r="G197">
+        <v>4</v>
+      </c>
       <c r="H197" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="198" spans="1:8" x14ac:dyDescent="0.25">
@@ -6033,7 +6237,7 @@
         <v>273</v>
       </c>
       <c r="C198" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D198" t="s">
         <v>284</v>
@@ -6041,8 +6245,14 @@
       <c r="E198" t="s">
         <v>278</v>
       </c>
+      <c r="F198">
+        <v>1</v>
+      </c>
+      <c r="G198">
+        <v>5</v>
+      </c>
       <c r="H198" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="199" spans="1:8" x14ac:dyDescent="0.25">
@@ -6053,7 +6263,7 @@
         <v>273</v>
       </c>
       <c r="C199" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D199" t="s">
         <v>284</v>
@@ -6061,8 +6271,14 @@
       <c r="E199" t="s">
         <v>279</v>
       </c>
+      <c r="F199">
+        <v>0</v>
+      </c>
+      <c r="G199">
+        <v>0</v>
+      </c>
       <c r="H199" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="200" spans="1:8" x14ac:dyDescent="0.25">
@@ -6073,7 +6289,7 @@
         <v>273</v>
       </c>
       <c r="C200" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="D200" t="s">
         <v>284</v>
@@ -6081,7 +6297,217 @@
       <c r="E200" t="s">
         <v>280</v>
       </c>
+      <c r="F200">
+        <v>0</v>
+      </c>
+      <c r="G200">
+        <v>1</v>
+      </c>
       <c r="H200" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="201" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A201">
+        <v>22</v>
+      </c>
+      <c r="B201" t="s">
+        <v>285</v>
+      </c>
+      <c r="D201" t="s">
+        <v>291</v>
+      </c>
+      <c r="E201" t="s">
+        <v>286</v>
+      </c>
+      <c r="H201" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="202" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A202">
+        <v>22</v>
+      </c>
+      <c r="B202" t="s">
+        <v>285</v>
+      </c>
+      <c r="D202" t="s">
+        <v>291</v>
+      </c>
+      <c r="E202" t="s">
+        <v>287</v>
+      </c>
+      <c r="H202" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="203" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A203">
+        <v>22</v>
+      </c>
+      <c r="B203" t="s">
+        <v>285</v>
+      </c>
+      <c r="D203" t="s">
+        <v>288</v>
+      </c>
+      <c r="E203" t="s">
+        <v>289</v>
+      </c>
+      <c r="H203" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="204" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A204">
+        <v>22</v>
+      </c>
+      <c r="B204" t="s">
+        <v>285</v>
+      </c>
+      <c r="D204" t="s">
+        <v>288</v>
+      </c>
+      <c r="E204" t="s">
+        <v>290</v>
+      </c>
+      <c r="H204" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="205" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A205">
+        <v>22</v>
+      </c>
+      <c r="B205" t="s">
+        <v>285</v>
+      </c>
+      <c r="D205" t="s">
+        <v>292</v>
+      </c>
+      <c r="E205" t="s">
+        <v>293</v>
+      </c>
+      <c r="H205" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="206" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A206">
+        <v>22</v>
+      </c>
+      <c r="B206" t="s">
+        <v>285</v>
+      </c>
+      <c r="D206" t="s">
+        <v>292</v>
+      </c>
+      <c r="E206" t="s">
+        <v>294</v>
+      </c>
+      <c r="H206" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="207" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A207">
+        <v>22</v>
+      </c>
+      <c r="B207" t="s">
+        <v>285</v>
+      </c>
+      <c r="D207" t="s">
+        <v>295</v>
+      </c>
+      <c r="E207" t="s">
+        <v>296</v>
+      </c>
+      <c r="H207" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="208" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A208">
+        <v>22</v>
+      </c>
+      <c r="B208" t="s">
+        <v>285</v>
+      </c>
+      <c r="D208" t="s">
+        <v>295</v>
+      </c>
+      <c r="E208" t="s">
+        <v>297</v>
+      </c>
+      <c r="H208" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="209" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A209">
+        <v>22</v>
+      </c>
+      <c r="B209" t="s">
+        <v>285</v>
+      </c>
+      <c r="D209" t="s">
+        <v>298</v>
+      </c>
+      <c r="E209" t="s">
+        <v>299</v>
+      </c>
+      <c r="H209" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="210" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A210">
+        <v>22</v>
+      </c>
+      <c r="B210" t="s">
+        <v>285</v>
+      </c>
+      <c r="D210" t="s">
+        <v>298</v>
+      </c>
+      <c r="E210" t="s">
+        <v>300</v>
+      </c>
+      <c r="H210" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="211" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A211">
+        <v>22</v>
+      </c>
+      <c r="B211" t="s">
+        <v>285</v>
+      </c>
+      <c r="D211" t="s">
+        <v>298</v>
+      </c>
+      <c r="E211" t="s">
+        <v>301</v>
+      </c>
+      <c r="H211" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="212" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A212">
+        <v>22</v>
+      </c>
+      <c r="B212" t="s">
+        <v>285</v>
+      </c>
+      <c r="D212" t="s">
+        <v>298</v>
+      </c>
+      <c r="E212" t="s">
+        <v>302</v>
+      </c>
+      <c r="H212" t="s">
         <v>149</v>
       </c>
     </row>

</xml_diff>

<commit_message>
labor of love results and gourd times questions
</commit_message>
<xml_diff>
--- a/whiteboardpollresults.xlsx
+++ b/whiteboardpollresults.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mbrownin\GitHub - Local\thehallwaypoll\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD209EB1-B4D5-4541-A45E-C12722BD993B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95AF389C-CBCD-4B1F-95EF-5AE36366AAE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="686" xr2:uid="{C0D0DBC0-4258-4C8D-AB0A-404DBED773F9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="325">
   <si>
     <t>option</t>
   </si>
@@ -945,6 +945,72 @@
   </si>
   <si>
     <t>Best</t>
+  </si>
+  <si>
+    <t>Moving Upward</t>
+  </si>
+  <si>
+    <t>Stairs</t>
+  </si>
+  <si>
+    <t>Elevator</t>
+  </si>
+  <si>
+    <t>Gourd Times</t>
+  </si>
+  <si>
+    <t>Favorite Leaf Color</t>
+  </si>
+  <si>
+    <t>Gold</t>
+  </si>
+  <si>
+    <t>Orange</t>
+  </si>
+  <si>
+    <t>Red</t>
+  </si>
+  <si>
+    <t>Ideal Field Trip</t>
+  </si>
+  <si>
+    <t>Apple Orchard</t>
+  </si>
+  <si>
+    <t>Corn Maze</t>
+  </si>
+  <si>
+    <t>Pumpkin Patch</t>
+  </si>
+  <si>
+    <t>Peak Fall Flavor</t>
+  </si>
+  <si>
+    <t>Pumpkin</t>
+  </si>
+  <si>
+    <t>Maple Pecan</t>
+  </si>
+  <si>
+    <t>Carmel Apple</t>
+  </si>
+  <si>
+    <t>Best Spice</t>
+  </si>
+  <si>
+    <t>Cloves</t>
+  </si>
+  <si>
+    <t>Ginger</t>
+  </si>
+  <si>
+    <t>Nutmeg</t>
+  </si>
+  <si>
+    <t>Décor Preference</t>
+  </si>
+  <si>
+    <t>Spooky</t>
   </si>
 </sst>
 </file>
@@ -1317,7 +1383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C897EEBF-8298-48F4-84CA-7840A621B809}">
-  <dimension ref="A1:H212"/>
+  <dimension ref="A1:H229"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
@@ -6314,14 +6380,23 @@
       <c r="B201" t="s">
         <v>285</v>
       </c>
+      <c r="C201" s="1">
+        <v>46293</v>
+      </c>
       <c r="D201" t="s">
         <v>291</v>
       </c>
       <c r="E201" t="s">
         <v>286</v>
       </c>
+      <c r="F201">
+        <v>21</v>
+      </c>
+      <c r="G201">
+        <v>0</v>
+      </c>
       <c r="H201" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="202" spans="1:8" x14ac:dyDescent="0.25">
@@ -6331,14 +6406,23 @@
       <c r="B202" t="s">
         <v>285</v>
       </c>
+      <c r="C202" s="1">
+        <v>46293</v>
+      </c>
       <c r="D202" t="s">
         <v>291</v>
       </c>
       <c r="E202" t="s">
         <v>287</v>
       </c>
+      <c r="F202">
+        <v>30</v>
+      </c>
+      <c r="G202">
+        <v>0</v>
+      </c>
       <c r="H202" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="203" spans="1:8" x14ac:dyDescent="0.25">
@@ -6348,14 +6432,23 @@
       <c r="B203" t="s">
         <v>285</v>
       </c>
+      <c r="C203" s="1">
+        <v>46293</v>
+      </c>
       <c r="D203" t="s">
-        <v>288</v>
+        <v>303</v>
       </c>
       <c r="E203" t="s">
-        <v>289</v>
+        <v>304</v>
+      </c>
+      <c r="F203">
+        <v>0</v>
+      </c>
+      <c r="G203">
+        <v>18</v>
       </c>
       <c r="H203" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="204" spans="1:8" x14ac:dyDescent="0.25">
@@ -6365,14 +6458,23 @@
       <c r="B204" t="s">
         <v>285</v>
       </c>
+      <c r="C204" s="1">
+        <v>46293</v>
+      </c>
       <c r="D204" t="s">
-        <v>288</v>
+        <v>303</v>
       </c>
       <c r="E204" t="s">
-        <v>290</v>
+        <v>305</v>
+      </c>
+      <c r="F204">
+        <v>0</v>
+      </c>
+      <c r="G204">
+        <v>16</v>
       </c>
       <c r="H204" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="205" spans="1:8" x14ac:dyDescent="0.25">
@@ -6382,14 +6484,23 @@
       <c r="B205" t="s">
         <v>285</v>
       </c>
+      <c r="C205" s="1">
+        <v>46293</v>
+      </c>
       <c r="D205" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="E205" t="s">
-        <v>293</v>
+        <v>289</v>
+      </c>
+      <c r="F205">
+        <v>20</v>
+      </c>
+      <c r="G205">
+        <v>16</v>
       </c>
       <c r="H205" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="206" spans="1:8" x14ac:dyDescent="0.25">
@@ -6399,14 +6510,23 @@
       <c r="B206" t="s">
         <v>285</v>
       </c>
+      <c r="C206" s="1">
+        <v>46293</v>
+      </c>
       <c r="D206" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="E206" t="s">
-        <v>294</v>
+        <v>290</v>
+      </c>
+      <c r="F206">
+        <v>39</v>
+      </c>
+      <c r="G206">
+        <v>17</v>
       </c>
       <c r="H206" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="207" spans="1:8" x14ac:dyDescent="0.25">
@@ -6416,14 +6536,23 @@
       <c r="B207" t="s">
         <v>285</v>
       </c>
+      <c r="C207" s="1">
+        <v>46293</v>
+      </c>
       <c r="D207" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E207" t="s">
-        <v>296</v>
+        <v>293</v>
+      </c>
+      <c r="F207">
+        <v>41</v>
+      </c>
+      <c r="G207">
+        <v>28</v>
       </c>
       <c r="H207" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="208" spans="1:8" x14ac:dyDescent="0.25">
@@ -6433,14 +6562,23 @@
       <c r="B208" t="s">
         <v>285</v>
       </c>
+      <c r="C208" s="1">
+        <v>46293</v>
+      </c>
       <c r="D208" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E208" t="s">
-        <v>297</v>
+        <v>294</v>
+      </c>
+      <c r="F208">
+        <v>16</v>
+      </c>
+      <c r="G208">
+        <v>5</v>
       </c>
       <c r="H208" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="209" spans="1:8" x14ac:dyDescent="0.25">
@@ -6450,14 +6588,23 @@
       <c r="B209" t="s">
         <v>285</v>
       </c>
+      <c r="C209" s="1">
+        <v>46293</v>
+      </c>
       <c r="D209" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="E209" t="s">
-        <v>299</v>
+        <v>296</v>
+      </c>
+      <c r="F209">
+        <v>45</v>
+      </c>
+      <c r="G209">
+        <v>23</v>
       </c>
       <c r="H209" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="210" spans="1:8" x14ac:dyDescent="0.25">
@@ -6467,14 +6614,23 @@
       <c r="B210" t="s">
         <v>285</v>
       </c>
+      <c r="C210" s="1">
+        <v>46293</v>
+      </c>
       <c r="D210" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="E210" t="s">
-        <v>300</v>
+        <v>297</v>
+      </c>
+      <c r="F210">
+        <v>14</v>
+      </c>
+      <c r="G210">
+        <v>11</v>
       </c>
       <c r="H210" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="211" spans="1:8" x14ac:dyDescent="0.25">
@@ -6484,14 +6640,23 @@
       <c r="B211" t="s">
         <v>285</v>
       </c>
+      <c r="C211" s="1">
+        <v>46293</v>
+      </c>
       <c r="D211" t="s">
         <v>298</v>
       </c>
       <c r="E211" t="s">
-        <v>301</v>
+        <v>299</v>
+      </c>
+      <c r="F211">
+        <v>36</v>
+      </c>
+      <c r="G211">
+        <v>22</v>
       </c>
       <c r="H211" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="212" spans="1:8" x14ac:dyDescent="0.25">
@@ -6501,13 +6666,329 @@
       <c r="B212" t="s">
         <v>285</v>
       </c>
+      <c r="C212" s="1">
+        <v>46293</v>
+      </c>
       <c r="D212" t="s">
         <v>298</v>
       </c>
       <c r="E212" t="s">
+        <v>300</v>
+      </c>
+      <c r="F212">
+        <v>4</v>
+      </c>
+      <c r="G212">
+        <v>2</v>
+      </c>
+      <c r="H212" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="213" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A213">
+        <v>22</v>
+      </c>
+      <c r="B213" t="s">
+        <v>285</v>
+      </c>
+      <c r="C213" s="1">
+        <v>46293</v>
+      </c>
+      <c r="D213" t="s">
+        <v>298</v>
+      </c>
+      <c r="E213" t="s">
+        <v>301</v>
+      </c>
+      <c r="F213">
+        <v>9</v>
+      </c>
+      <c r="G213">
+        <v>10</v>
+      </c>
+      <c r="H213" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="214" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A214">
+        <v>22</v>
+      </c>
+      <c r="B214" t="s">
+        <v>285</v>
+      </c>
+      <c r="C214" s="1">
+        <v>46293</v>
+      </c>
+      <c r="D214" t="s">
+        <v>298</v>
+      </c>
+      <c r="E214" t="s">
         <v>302</v>
       </c>
-      <c r="H212" t="s">
+      <c r="F214">
+        <v>25</v>
+      </c>
+      <c r="G214">
+        <v>10</v>
+      </c>
+      <c r="H214" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="215" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A215">
+        <v>23</v>
+      </c>
+      <c r="B215" t="s">
+        <v>306</v>
+      </c>
+      <c r="D215" t="s">
+        <v>307</v>
+      </c>
+      <c r="E215" t="s">
+        <v>308</v>
+      </c>
+      <c r="H215" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="216" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A216">
+        <v>23</v>
+      </c>
+      <c r="B216" t="s">
+        <v>306</v>
+      </c>
+      <c r="D216" t="s">
+        <v>307</v>
+      </c>
+      <c r="E216" t="s">
+        <v>309</v>
+      </c>
+      <c r="H216" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="217" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A217">
+        <v>23</v>
+      </c>
+      <c r="B217" t="s">
+        <v>306</v>
+      </c>
+      <c r="D217" t="s">
+        <v>307</v>
+      </c>
+      <c r="E217" t="s">
+        <v>310</v>
+      </c>
+      <c r="H217" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="218" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A218">
+        <v>23</v>
+      </c>
+      <c r="B218" t="s">
+        <v>306</v>
+      </c>
+      <c r="D218" t="s">
+        <v>311</v>
+      </c>
+      <c r="E218" t="s">
+        <v>312</v>
+      </c>
+      <c r="H218" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="219" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A219">
+        <v>23</v>
+      </c>
+      <c r="B219" t="s">
+        <v>306</v>
+      </c>
+      <c r="D219" t="s">
+        <v>311</v>
+      </c>
+      <c r="E219" t="s">
+        <v>313</v>
+      </c>
+      <c r="H219" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="220" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A220">
+        <v>23</v>
+      </c>
+      <c r="B220" t="s">
+        <v>306</v>
+      </c>
+      <c r="D220" t="s">
+        <v>311</v>
+      </c>
+      <c r="E220" t="s">
+        <v>314</v>
+      </c>
+      <c r="H220" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="221" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A221">
+        <v>23</v>
+      </c>
+      <c r="B221" t="s">
+        <v>306</v>
+      </c>
+      <c r="D221" t="s">
+        <v>315</v>
+      </c>
+      <c r="E221" t="s">
+        <v>316</v>
+      </c>
+      <c r="H221" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="222" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A222">
+        <v>23</v>
+      </c>
+      <c r="B222" t="s">
+        <v>306</v>
+      </c>
+      <c r="D222" t="s">
+        <v>315</v>
+      </c>
+      <c r="E222" t="s">
+        <v>317</v>
+      </c>
+      <c r="H222" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="223" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A223">
+        <v>23</v>
+      </c>
+      <c r="B223" t="s">
+        <v>306</v>
+      </c>
+      <c r="D223" t="s">
+        <v>315</v>
+      </c>
+      <c r="E223" t="s">
+        <v>318</v>
+      </c>
+      <c r="H223" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="224" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A224">
+        <v>23</v>
+      </c>
+      <c r="B224" t="s">
+        <v>306</v>
+      </c>
+      <c r="D224" t="s">
+        <v>319</v>
+      </c>
+      <c r="E224" t="s">
+        <v>208</v>
+      </c>
+      <c r="H224" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="225" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A225">
+        <v>23</v>
+      </c>
+      <c r="B225" t="s">
+        <v>306</v>
+      </c>
+      <c r="D225" t="s">
+        <v>319</v>
+      </c>
+      <c r="E225" t="s">
+        <v>320</v>
+      </c>
+      <c r="H225" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="226" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A226">
+        <v>23</v>
+      </c>
+      <c r="B226" t="s">
+        <v>306</v>
+      </c>
+      <c r="D226" t="s">
+        <v>319</v>
+      </c>
+      <c r="E226" t="s">
+        <v>321</v>
+      </c>
+      <c r="H226" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="227" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A227">
+        <v>23</v>
+      </c>
+      <c r="B227" t="s">
+        <v>306</v>
+      </c>
+      <c r="D227" t="s">
+        <v>319</v>
+      </c>
+      <c r="E227" t="s">
+        <v>322</v>
+      </c>
+      <c r="H227" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="228" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A228">
+        <v>23</v>
+      </c>
+      <c r="B228" t="s">
+        <v>306</v>
+      </c>
+      <c r="D228" t="s">
+        <v>323</v>
+      </c>
+      <c r="E228" t="s">
+        <v>30</v>
+      </c>
+      <c r="H228" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="229" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A229">
+        <v>23</v>
+      </c>
+      <c r="B229" t="s">
+        <v>306</v>
+      </c>
+      <c r="D229" t="s">
+        <v>323</v>
+      </c>
+      <c r="E229" t="s">
+        <v>324</v>
+      </c>
+      <c r="H229" t="s">
         <v>149</v>
       </c>
     </row>

</xml_diff>

<commit_message>
labor of love post and gourd times results update
</commit_message>
<xml_diff>
--- a/whiteboardpollresults.xlsx
+++ b/whiteboardpollresults.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mbrownin\GitHub - Local\thehallwaypoll\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95AF389C-CBCD-4B1F-95EF-5AE36366AAE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FF608E2-2FEE-44F6-868D-0F8422A88AA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="686" xr2:uid="{C0D0DBC0-4258-4C8D-AB0A-404DBED773F9}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="686" xr2:uid="{C0D0DBC0-4258-4C8D-AB0A-404DBED773F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="960" uniqueCount="337">
   <si>
     <t>option</t>
   </si>
@@ -1011,6 +1011,42 @@
   </si>
   <si>
     <t>Spooky</t>
+  </si>
+  <si>
+    <t>Trick or Treat?</t>
+  </si>
+  <si>
+    <t>Costume</t>
+  </si>
+  <si>
+    <t>Handemade</t>
+  </si>
+  <si>
+    <t>Store-bought</t>
+  </si>
+  <si>
+    <t>Scary</t>
+  </si>
+  <si>
+    <t>Candy</t>
+  </si>
+  <si>
+    <t>Chocolate</t>
+  </si>
+  <si>
+    <t>Gummy</t>
+  </si>
+  <si>
+    <t>Trick-or-treat Stash</t>
+  </si>
+  <si>
+    <t>Savor as long as you can</t>
+  </si>
+  <si>
+    <t>Gorge it quickly</t>
+  </si>
+  <si>
+    <t>Carving Pumpkins</t>
   </si>
 </sst>
 </file>
@@ -1383,7 +1419,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C897EEBF-8298-48F4-84CA-7840A621B809}">
-  <dimension ref="A1:H229"/>
+  <dimension ref="A1:H239"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
@@ -6744,14 +6780,23 @@
       <c r="B215" t="s">
         <v>306</v>
       </c>
+      <c r="C215" s="1">
+        <v>46321</v>
+      </c>
       <c r="D215" t="s">
         <v>307</v>
       </c>
       <c r="E215" t="s">
         <v>308</v>
       </c>
+      <c r="F215">
+        <v>13</v>
+      </c>
+      <c r="G215">
+        <v>28</v>
+      </c>
       <c r="H215" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="216" spans="1:8" x14ac:dyDescent="0.25">
@@ -6761,14 +6806,23 @@
       <c r="B216" t="s">
         <v>306</v>
       </c>
+      <c r="C216" s="1">
+        <v>46321</v>
+      </c>
       <c r="D216" t="s">
         <v>307</v>
       </c>
       <c r="E216" t="s">
         <v>309</v>
       </c>
+      <c r="F216">
+        <v>17</v>
+      </c>
+      <c r="G216">
+        <v>9</v>
+      </c>
       <c r="H216" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="217" spans="1:8" x14ac:dyDescent="0.25">
@@ -6778,14 +6832,23 @@
       <c r="B217" t="s">
         <v>306</v>
       </c>
+      <c r="C217" s="1">
+        <v>46321</v>
+      </c>
       <c r="D217" t="s">
         <v>307</v>
       </c>
       <c r="E217" t="s">
         <v>310</v>
       </c>
+      <c r="F217">
+        <v>37</v>
+      </c>
+      <c r="G217">
+        <v>19</v>
+      </c>
       <c r="H217" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="218" spans="1:8" x14ac:dyDescent="0.25">
@@ -6795,14 +6858,23 @@
       <c r="B218" t="s">
         <v>306</v>
       </c>
+      <c r="C218" s="1">
+        <v>46321</v>
+      </c>
       <c r="D218" t="s">
         <v>311</v>
       </c>
       <c r="E218" t="s">
         <v>312</v>
       </c>
+      <c r="F218">
+        <v>38</v>
+      </c>
+      <c r="G218">
+        <v>15</v>
+      </c>
       <c r="H218" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="219" spans="1:8" x14ac:dyDescent="0.25">
@@ -6812,14 +6884,23 @@
       <c r="B219" t="s">
         <v>306</v>
       </c>
+      <c r="C219" s="1">
+        <v>46321</v>
+      </c>
       <c r="D219" t="s">
         <v>311</v>
       </c>
       <c r="E219" t="s">
         <v>313</v>
       </c>
+      <c r="F219">
+        <v>9</v>
+      </c>
+      <c r="G219">
+        <v>1</v>
+      </c>
       <c r="H219" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="220" spans="1:8" x14ac:dyDescent="0.25">
@@ -6829,14 +6910,23 @@
       <c r="B220" t="s">
         <v>306</v>
       </c>
+      <c r="C220" s="1">
+        <v>46321</v>
+      </c>
       <c r="D220" t="s">
         <v>311</v>
       </c>
       <c r="E220" t="s">
         <v>314</v>
       </c>
+      <c r="F220">
+        <v>19</v>
+      </c>
+      <c r="G220">
+        <v>9</v>
+      </c>
       <c r="H220" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="221" spans="1:8" x14ac:dyDescent="0.25">
@@ -6846,14 +6936,23 @@
       <c r="B221" t="s">
         <v>306</v>
       </c>
+      <c r="C221" s="1">
+        <v>46321</v>
+      </c>
       <c r="D221" t="s">
         <v>315</v>
       </c>
       <c r="E221" t="s">
         <v>316</v>
       </c>
+      <c r="F221">
+        <v>22</v>
+      </c>
+      <c r="G221">
+        <v>16</v>
+      </c>
       <c r="H221" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="222" spans="1:8" x14ac:dyDescent="0.25">
@@ -6863,14 +6962,23 @@
       <c r="B222" t="s">
         <v>306</v>
       </c>
+      <c r="C222" s="1">
+        <v>46321</v>
+      </c>
       <c r="D222" t="s">
         <v>315</v>
       </c>
       <c r="E222" t="s">
         <v>317</v>
       </c>
+      <c r="F222">
+        <v>22</v>
+      </c>
+      <c r="G222">
+        <v>13</v>
+      </c>
       <c r="H222" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="223" spans="1:8" x14ac:dyDescent="0.25">
@@ -6880,14 +6988,23 @@
       <c r="B223" t="s">
         <v>306</v>
       </c>
+      <c r="C223" s="1">
+        <v>46321</v>
+      </c>
       <c r="D223" t="s">
         <v>315</v>
       </c>
       <c r="E223" t="s">
         <v>318</v>
       </c>
+      <c r="F223">
+        <v>20</v>
+      </c>
+      <c r="G223">
+        <v>6</v>
+      </c>
       <c r="H223" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="224" spans="1:8" x14ac:dyDescent="0.25">
@@ -6897,14 +7014,23 @@
       <c r="B224" t="s">
         <v>306</v>
       </c>
+      <c r="C224" s="1">
+        <v>46321</v>
+      </c>
       <c r="D224" t="s">
         <v>319</v>
       </c>
       <c r="E224" t="s">
         <v>208</v>
       </c>
+      <c r="F224">
+        <v>37</v>
+      </c>
+      <c r="G224">
+        <v>21</v>
+      </c>
       <c r="H224" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="225" spans="1:8" x14ac:dyDescent="0.25">
@@ -6914,14 +7040,23 @@
       <c r="B225" t="s">
         <v>306</v>
       </c>
+      <c r="C225" s="1">
+        <v>46321</v>
+      </c>
       <c r="D225" t="s">
         <v>319</v>
       </c>
       <c r="E225" t="s">
         <v>320</v>
       </c>
+      <c r="F225">
+        <v>6</v>
+      </c>
+      <c r="G225">
+        <v>8</v>
+      </c>
       <c r="H225" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="226" spans="1:8" x14ac:dyDescent="0.25">
@@ -6931,14 +7066,23 @@
       <c r="B226" t="s">
         <v>306</v>
       </c>
+      <c r="C226" s="1">
+        <v>46321</v>
+      </c>
       <c r="D226" t="s">
         <v>319</v>
       </c>
       <c r="E226" t="s">
         <v>321</v>
       </c>
+      <c r="F226">
+        <v>14</v>
+      </c>
+      <c r="G226">
+        <v>7</v>
+      </c>
       <c r="H226" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="227" spans="1:8" x14ac:dyDescent="0.25">
@@ -6948,14 +7092,23 @@
       <c r="B227" t="s">
         <v>306</v>
       </c>
+      <c r="C227" s="1">
+        <v>46321</v>
+      </c>
       <c r="D227" t="s">
         <v>319</v>
       </c>
       <c r="E227" t="s">
         <v>322</v>
       </c>
+      <c r="F227">
+        <v>9</v>
+      </c>
+      <c r="G227">
+        <v>2</v>
+      </c>
       <c r="H227" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="228" spans="1:8" x14ac:dyDescent="0.25">
@@ -6965,14 +7118,23 @@
       <c r="B228" t="s">
         <v>306</v>
       </c>
+      <c r="C228" s="1">
+        <v>46321</v>
+      </c>
       <c r="D228" t="s">
         <v>323</v>
       </c>
       <c r="E228" t="s">
         <v>30</v>
       </c>
+      <c r="F228">
+        <v>53</v>
+      </c>
+      <c r="G228">
+        <v>25</v>
+      </c>
       <c r="H228" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="229" spans="1:8" x14ac:dyDescent="0.25">
@@ -6982,13 +7144,222 @@
       <c r="B229" t="s">
         <v>306</v>
       </c>
+      <c r="C229" s="1">
+        <v>46321</v>
+      </c>
       <c r="D229" t="s">
         <v>323</v>
       </c>
       <c r="E229" t="s">
         <v>324</v>
       </c>
+      <c r="F229">
+        <v>14</v>
+      </c>
+      <c r="G229">
+        <v>14</v>
+      </c>
       <c r="H229" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="230" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A230">
+        <v>24</v>
+      </c>
+      <c r="B230" t="s">
+        <v>325</v>
+      </c>
+      <c r="C230" s="1">
+        <v>46328</v>
+      </c>
+      <c r="D230" t="s">
+        <v>326</v>
+      </c>
+      <c r="E230" t="s">
+        <v>327</v>
+      </c>
+      <c r="H230" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="231" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A231">
+        <v>24</v>
+      </c>
+      <c r="B231" t="s">
+        <v>325</v>
+      </c>
+      <c r="C231" s="1">
+        <v>46328</v>
+      </c>
+      <c r="D231" t="s">
+        <v>326</v>
+      </c>
+      <c r="E231" t="s">
+        <v>328</v>
+      </c>
+      <c r="H231" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="232" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A232">
+        <v>24</v>
+      </c>
+      <c r="B232" t="s">
+        <v>325</v>
+      </c>
+      <c r="C232" s="1">
+        <v>46328</v>
+      </c>
+      <c r="D232" t="s">
+        <v>98</v>
+      </c>
+      <c r="E232" t="s">
+        <v>324</v>
+      </c>
+      <c r="H232" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="233" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A233">
+        <v>24</v>
+      </c>
+      <c r="B233" t="s">
+        <v>325</v>
+      </c>
+      <c r="C233" s="1">
+        <v>46328</v>
+      </c>
+      <c r="D233" t="s">
+        <v>98</v>
+      </c>
+      <c r="E233" t="s">
+        <v>329</v>
+      </c>
+      <c r="H233" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="234" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A234">
+        <v>24</v>
+      </c>
+      <c r="B234" t="s">
+        <v>325</v>
+      </c>
+      <c r="C234" s="1">
+        <v>46328</v>
+      </c>
+      <c r="D234" t="s">
+        <v>330</v>
+      </c>
+      <c r="E234" t="s">
+        <v>331</v>
+      </c>
+      <c r="H234" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="235" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A235">
+        <v>24</v>
+      </c>
+      <c r="B235" t="s">
+        <v>325</v>
+      </c>
+      <c r="C235" s="1">
+        <v>46328</v>
+      </c>
+      <c r="D235" t="s">
+        <v>330</v>
+      </c>
+      <c r="E235" t="s">
+        <v>332</v>
+      </c>
+      <c r="H235" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="236" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A236">
+        <v>24</v>
+      </c>
+      <c r="B236" t="s">
+        <v>325</v>
+      </c>
+      <c r="C236" s="1">
+        <v>46328</v>
+      </c>
+      <c r="D236" t="s">
+        <v>333</v>
+      </c>
+      <c r="E236" t="s">
+        <v>334</v>
+      </c>
+      <c r="H236" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="237" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A237">
+        <v>24</v>
+      </c>
+      <c r="B237" t="s">
+        <v>325</v>
+      </c>
+      <c r="C237" s="1">
+        <v>46328</v>
+      </c>
+      <c r="D237" t="s">
+        <v>333</v>
+      </c>
+      <c r="E237" t="s">
+        <v>335</v>
+      </c>
+      <c r="H237" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="238" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A238">
+        <v>24</v>
+      </c>
+      <c r="B238" t="s">
+        <v>325</v>
+      </c>
+      <c r="C238" s="1">
+        <v>46328</v>
+      </c>
+      <c r="D238" t="s">
+        <v>336</v>
+      </c>
+      <c r="E238" t="s">
+        <v>236</v>
+      </c>
+      <c r="H238" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="239" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A239">
+        <v>24</v>
+      </c>
+      <c r="B239" t="s">
+        <v>325</v>
+      </c>
+      <c r="C239" s="1">
+        <v>46328</v>
+      </c>
+      <c r="D239" t="s">
+        <v>336</v>
+      </c>
+      <c r="E239" t="s">
+        <v>237</v>
+      </c>
+      <c r="H239" t="s">
         <v>149</v>
       </c>
     </row>

</xml_diff>